<commit_message>
Overhauled all pages with production level quality design, bug fixes.
</commit_message>
<xml_diff>
--- a/Unit testing Calorific.xlsx
+++ b/Unit testing Calorific.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mlmda\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ucf-my.sharepoint.com/personal/sh191143_ucf_edu/Documents/Projects/Calorific/Calorific/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A15A98A3-1E61-4876-B7EC-116637EBBCF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="8_{A15A98A3-1E61-4876-B7EC-116637EBBCF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4C31BE4C-AF60-4EBF-9BBF-2C76BB34C2EC}"/>
   <bookViews>
-    <workbookView xWindow="390" yWindow="390" windowWidth="21600" windowHeight="11385" xr2:uid="{5101CC7E-5DFC-49A3-814E-81BE405B7B7E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{5101CC7E-5DFC-49A3-814E-81BE405B7B7E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -152,7 +152,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -296,6 +296,185 @@
         </a:extLst>
       </xdr:spPr>
     </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>176892</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>489857</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>517586</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>976002</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8277CCBD-D06F-DB26-2FA2-9E9CF51B2FD7}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9443356" y="870857"/>
+          <a:ext cx="3402301" cy="4772395"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>139052</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>489858</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>40374</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>1004209</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1F35C8DB-858F-0FF0-D6A9-EE955C6EFBBE}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="13079445" y="870858"/>
+          <a:ext cx="3575250" cy="4800601"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>216538</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>489857</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>100884</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>1004208</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4C3B3638-B1ED-56F9-A12E-67EC04FDCAB5}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="16830859" y="870857"/>
+          <a:ext cx="3558275" cy="4800601"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>299356</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>1088571</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>118220</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>34650</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0CB903D6-382E-B542-9376-FD77828EF268}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="10178142" y="5755821"/>
+          <a:ext cx="9003685" cy="5409472"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:effectLst>
+          <a:softEdge rad="31750"/>
+        </a:effectLst>
+      </xdr:spPr>
+    </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
@@ -728,13 +907,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C5A8132-7A67-49B1-BD59-755C4DD3F028}">
   <dimension ref="B3:C7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="59.7109375" customWidth="1"/>
     <col min="3" max="3" width="70" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:3" ht="203.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:3" ht="203.25" customHeight="1">
       <c r="B3" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
@@ -742,7 +921,7 @@
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="4" spans="2:3" ht="134.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:3" ht="134.25" customHeight="1">
       <c r="B4" t="e" vm="3">
         <v>#VALUE!</v>
       </c>
@@ -750,7 +929,7 @@
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="5" spans="2:3" ht="134.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:3" ht="134.25" customHeight="1">
       <c r="B5" t="e" vm="5">
         <v>#VALUE!</v>
       </c>
@@ -758,7 +937,7 @@
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="6" spans="2:3" ht="149.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:3" ht="149.25" customHeight="1">
       <c r="B6" t="e" vm="7">
         <v>#VALUE!</v>
       </c>
@@ -766,7 +945,7 @@
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="7" spans="2:3" ht="120.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:3" ht="120.75" customHeight="1">
       <c r="B7" t="e" vm="9">
         <v>#VALUE!</v>
       </c>

</xml_diff>